<commit_message>
feat(digs): finish demo package targets
</commit_message>
<xml_diff>
--- a/qa/VOX_QA_FEEDBACK.xlsx
+++ b/qa/VOX_QA_FEEDBACK.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checkpoints'!$A$1:$N$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Issues'!$A$1:$O$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Environment'!$A$1:$D$51</definedName>
   </definedNames>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N103"/>
+  <dimension ref="A1:N115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5868,9 +5868,633 @@
       <c r="M103" s="3" t="inlineStr"/>
       <c r="N103" s="3" t="inlineStr"/>
     </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-105</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Fluids</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Dam and channel retain and release water</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Start PRACTICE with HYDROSHOT and make a sloped channel ending in a solid dam</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Fill the channel; wait for leveling; breach the dam; repeat with a large sustained stream</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Water pools upstream; crossing the breach makes a downhill stream; a full fluid pool does not freeze falling water or delete a failed deposit</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Video before and after breach; candidate checksum; conservation and capacity self-test output</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr"/>
+      <c r="K104" s="3" t="inlineStr"/>
+      <c r="L104" s="3" t="inlineStr"/>
+      <c r="M104" s="3" t="inlineStr"/>
+      <c r="N104" s="3" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-106</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Fluids</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Magma and blood remain physical volumes</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Open a magma pocket and create several projectile kills above a downhill basin</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Observe the lava spill; use water at its edge; observe blood collection and run-off</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Lava flows from its opening and reacts with water; blood lands and gathers downhill; effects remain readable and do not create invisible solid collisions</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Video of each material and reaction with map and candidate checksum</t>
+        </is>
+      </c>
+      <c r="H105" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J105" s="3" t="inlineStr"/>
+      <c r="K105" s="3" t="inlineStr"/>
+      <c r="L105" s="3" t="inlineStr"/>
+      <c r="M105" s="3" t="inlineStr"/>
+      <c r="N105" s="3" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-107</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Gameplay</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Shallow water is safe and immersion drowns</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Make a shallow pool and a head-deep water or blood basin</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Stand in the shallow pool; submerge the head; escape with Steam Hook or steam; observe bot escapes</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Foot-level liquid does not cause drowning; actual head immersion causes damage; escape stops drowning; bots react to immersion</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>Video with health before during and after immersion; drowning self-test output</t>
+        </is>
+      </c>
+      <c r="H106" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J106" s="3" t="inlineStr"/>
+      <c r="K106" s="3" t="inlineStr"/>
+      <c r="L106" s="3" t="inlineStr"/>
+      <c r="M106" s="3" t="inlineStr"/>
+      <c r="N106" s="3" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-108</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Terrain</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Connected support reaches genuine anchors</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Build or locate a broad overhang and a tall column connected to ground; keep a miner away from the debris path</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Cut one local underside while remote supports remain; remove the final connection; repeat on a structure larger than one debris fragment</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>A genuine remote support holds connected terrain; a floating column is not its own anchor; detached groups collapse through bounded fragments without a disappearing whole roof or an unbounded stall</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Video showing last support and resulting debris; connected-component self-test output</t>
+        </is>
+      </c>
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J107" s="3" t="inlineStr"/>
+      <c r="K107" s="3" t="inlineStr"/>
+      <c r="L107" s="3" t="inlineStr"/>
+      <c r="M107" s="3" t="inlineStr"/>
+      <c r="N107" s="3" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-109</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Anatomy</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Damage class decides the death</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Use all direct projectile and melee weapons plus explosive and heat kills</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>Observe entry-point severing; compare low-power POPPER limb damage with FIRECRACKER blast and lava deaths; land a headshot</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Direct kills sever from impact; low-power bullets do not routinely disconnect every body part; blasts disconnect and heat melts; headshots display their distinct award</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Video per damage class with weapon and candidate checksum; death-policy self-test output</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J108" s="3" t="inlineStr"/>
+      <c r="K108" s="3" t="inlineStr"/>
+      <c r="L108" s="3" t="inlineStr"/>
+      <c r="M108" s="3" t="inlineStr"/>
+      <c r="N108" s="3" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-110</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>All eleven tools have distinct carried models</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Enable Full Works and aim at terrain in PRACTICE</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Cycle all eleven weapons; aim left right up and down; fire or charge each</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Carried silhouettes are distinct and face the aim; projectile muzzle flashes and smoke begin at the weapon; melee tools read as their intended forms</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Contact sheet or video of eleven tools and their muzzle positions</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="inlineStr"/>
+      <c r="K109" s="3" t="inlineStr"/>
+      <c r="L109" s="3" t="inlineStr"/>
+      <c r="M109" s="3" t="inlineStr"/>
+      <c r="N109" s="3" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-111</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Articulated miners move through all poses</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Play with a human miner and all three bots</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>Walk jump steam fire and take a survivable hit; observe corpses separately</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Connected limb segments produce readable walk jump steam pain and fire poses; joints do not leave limbs floating; motion does not change collision or replay state</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Video of all poses; articulated-pose and render-hash regression output</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr"/>
+      <c r="K110" s="3" t="inlineStr"/>
+      <c r="L110" s="3" t="inlineStr"/>
+      <c r="M110" s="3" t="inlineStr"/>
+      <c r="N110" s="3" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-112</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Background depth preserves material clarity</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Visit Coal Ridge Deepworks and Furnace Yard at close and wide zoom</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Pan through each map; compare atmosphere across Lightfield tiers and Laptop Mode</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Background terrain layers move with parallax; bounded cloud volume and white moon stay behind air; neither paints over occupied terrain or hides live debris</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Screenshots and video at each map and representative zoom</t>
+        </is>
+      </c>
+      <c r="H111" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J111" s="3" t="inlineStr"/>
+      <c r="K111" s="3" t="inlineStr"/>
+      <c r="L111" s="3" t="inlineStr"/>
+      <c r="M111" s="3" t="inlineStr"/>
+      <c r="N111" s="3" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-113</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Weapon camera movement remains controllable</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Play at low and high supported frame caps in a one-human and two-human match</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>Move; use close weapons; charge throw and Railshot; die; watch the best-kill replay</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Camera pull sway release and death zoom are subtle; Railshot charge leads toward aim; both local miners stay framed; replay pacing preserves the selected exchange</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>Video and cap settings; camera and replay self-test output</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J112" s="3" t="inlineStr"/>
+      <c r="K112" s="3" t="inlineStr"/>
+      <c r="L112" s="3" t="inlineStr"/>
+      <c r="M112" s="3" t="inlineStr"/>
+      <c r="N112" s="3" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-114</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Speech and death sounds identify each miner</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Enable audio and play with RIVET CINDER and FLAMEY</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>Hear conversation; cause several damage-type deaths and survivable hits; repeat with audio unavailable</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>Phonetic articulation remains intelligible in the chosen style; death moans and pain grunts are audible and distinct; silence fallback preserves gameplay</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>Audio or video with voice settings; audio deterministic self-test output</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr"/>
+      <c r="K113" s="3" t="inlineStr"/>
+      <c r="L113" s="3" t="inlineStr"/>
+      <c r="M113" s="3" t="inlineStr"/>
+      <c r="N113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-115</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Five-minute destruction records actual service timing</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>Use the exact candidate on the named bench with ordinary background load recorded</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>Run digs_demo --performance-stress-self-test; retain complete output and exit status; separately perform VOX-QA-084</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>The 18000-tick lane reports measured p99 maximum final and peak virtual service debt and late ticks; p99 is at most 16.67 ms and final service debt is zero; this is simulation timing and does not replace the human soak</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>Raw stdout stderr exit status CPU power state compiler and candidate SHA-256</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J114" s="3" t="inlineStr"/>
+      <c r="K114" s="3" t="inlineStr"/>
+      <c r="L114" s="3" t="inlineStr"/>
+      <c r="M114" s="3" t="inlineStr"/>
+      <c r="N114" s="3" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>VOX-QA-116</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Extracted-package results are shipped and hashed</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>Extract the candidate binary and Corresponding Source archives into fresh directories</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>Verify SHA256SUMS; inspect packaged-input load and smoke stdout stderr exit files; verify their SBOM checksums; rebuild the source</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>All extracted-package evidence is present in the delivered archive; every successful exit is recorded as zero; source corresponds to the executable and playable payload stays within its ceiling</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>Checksum verification source rebuild output and SBOM file-check report</t>
+        </is>
+      </c>
+      <c r="H115" s="3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="J115" s="3" t="inlineStr"/>
+      <c r="K115" s="3" t="inlineStr"/>
+      <c r="L115" s="3" t="inlineStr"/>
+      <c r="M115" s="3" t="inlineStr"/>
+      <c r="N115" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N103"/>
-  <conditionalFormatting sqref="H2:H103">
+  <autoFilter ref="A1:N115"/>
+  <conditionalFormatting sqref="H2:H115">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>H2="Pass"</formula>
     </cfRule>
@@ -5882,10 +6506,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="H2:H103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
+    <dataValidation sqref="H2:H115" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Record the checkpoint outcome." type="list" errorStyle="stop">
       <formula1>"Not Run,Pass,Fail,Blocked,Skip"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I103" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
+    <dataValidation sqref="I2:I115" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid QA value" error="Choose a value from the list." promptTitle="VOX QA" prompt="Choose impact only when the result is Fail or Blocked." type="list" errorStyle="stop">
       <formula1>"NOTE,LOW,MEDIUM,HIGH,BLOCKER"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>